<commit_message>
fix(7013): SOTP model — Sensitivity layout, Peer font consistency
1. Sensitivity: B column widened from 22 to 38 for full label visibility
2. Peer Comps: font styles unified across all 4 segment blocks
   - Included peers: Company 10pt black, Ticker 10pt gray, values 10pt blue, Note 9pt gray
   - Excluded peer (TransDigm): all columns gray italic
   - Ticker column standardized from 9pt to 10pt

Verified: recalc.py PASS, 0 errors, 0 warnings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/7013_SOTP_Model.xlsx
+++ b/models/7013_SOTP_Model.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="167" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +75,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
       <sz val="10"/>
     </font>
     <font>
@@ -165,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -194,18 +210,21 @@
     <xf numFmtId="165" fontId="5" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="8" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,7 +244,7 @@
     <xf numFmtId="166" fontId="8" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1207,7 +1226,7 @@
       <c r="F5" s="23" t="n">
         <v>130</v>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>CFM LEAP, MRO, Defense</t>
         </is>
@@ -1233,7 +1252,7 @@
       <c r="F6" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="24" t="inlineStr">
         <is>
           <t>V2500/PW1100G partner</t>
         </is>
@@ -1259,70 +1278,70 @@
       <c r="F7" s="23" t="n">
         <v>65</v>
       </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Large engine, V-shape recovery</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>TransDigm</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>TDG</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="27" t="n">
         <v>0.54</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="28" t="n">
         <v>75</v>
       </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Aftermarket monopoly — EXCLUDED</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr"/>
-      <c r="D9" s="29">
+      <c r="C9" s="31" t="inlineStr"/>
+      <c r="D9" s="32">
         <f>MEDIAN(D5,D6,D7)</f>
         <v/>
       </c>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="28" t="inlineStr"/>
-      <c r="G9" s="28" t="inlineStr"/>
+      <c r="E9" s="31" t="inlineStr"/>
+      <c r="F9" s="31" t="inlineStr"/>
+      <c r="G9" s="31" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Selected Multiple</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="34" t="inlineStr">
         <is>
           <t>Median of Safran/MTU/Rolls-Royce (excl. TransDigm)</t>
         </is>
       </c>
-      <c r="D10" s="32" t="n">
+      <c r="D10" s="35" t="n">
         <v>18</v>
       </c>
-      <c r="E10" s="33" t="inlineStr"/>
-      <c r="F10" s="33" t="inlineStr"/>
-      <c r="G10" s="33" t="inlineStr"/>
+      <c r="E10" s="36" t="inlineStr"/>
+      <c r="F10" s="36" t="inlineStr"/>
+      <c r="G10" s="36" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="18" t="inlineStr">
@@ -1388,7 +1407,7 @@
       <c r="F14" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="24" t="inlineStr">
         <is>
           <t>Gas turbine, grid</t>
         </is>
@@ -1414,44 +1433,44 @@
       <c r="F15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="G15" s="24" t="inlineStr">
         <is>
           <t>Comparable segment estimate</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr"/>
-      <c r="D16" s="29">
+      <c r="C16" s="31" t="inlineStr"/>
+      <c r="D16" s="32">
         <f>MEDIAN(D14,D15)</f>
         <v/>
       </c>
-      <c r="E16" s="28" t="inlineStr"/>
-      <c r="F16" s="28" t="inlineStr"/>
-      <c r="G16" s="28" t="inlineStr"/>
+      <c r="E16" s="31" t="inlineStr"/>
+      <c r="F16" s="31" t="inlineStr"/>
+      <c r="G16" s="31" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="33" t="inlineStr">
         <is>
           <t>Selected Multiple</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="34" t="inlineStr">
         <is>
           <t>Energy equipment peers</t>
         </is>
       </c>
-      <c r="D17" s="32" t="n">
+      <c r="D17" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="E17" s="33" t="inlineStr"/>
-      <c r="F17" s="33" t="inlineStr"/>
-      <c r="G17" s="33" t="inlineStr"/>
+      <c r="E17" s="36" t="inlineStr"/>
+      <c r="F17" s="36" t="inlineStr"/>
+      <c r="G17" s="36" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="18" t="inlineStr">
@@ -1517,7 +1536,7 @@
       <c r="F21" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="G21" s="24" t="inlineStr">
         <is>
           <t>Turbocharger OEM</t>
         </is>
@@ -1543,44 +1562,44 @@
       <c r="F22" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="20" t="inlineStr">
+      <c r="G22" s="24" t="inlineStr">
         <is>
           <t>Turbocharger pure-play</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr"/>
-      <c r="D23" s="29">
+      <c r="C23" s="31" t="inlineStr"/>
+      <c r="D23" s="32">
         <f>MEDIAN(D21,D22)</f>
         <v/>
       </c>
-      <c r="E23" s="28" t="inlineStr"/>
-      <c r="F23" s="28" t="inlineStr"/>
-      <c r="G23" s="28" t="inlineStr"/>
+      <c r="E23" s="31" t="inlineStr"/>
+      <c r="F23" s="31" t="inlineStr"/>
+      <c r="G23" s="31" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
         <is>
           <t>Selected Multiple</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="34" t="inlineStr">
         <is>
           <t>Turbocharger/machinery blend</t>
         </is>
       </c>
-      <c r="D24" s="32" t="n">
+      <c r="D24" s="35" t="n">
         <v>10</v>
       </c>
-      <c r="E24" s="33" t="inlineStr"/>
-      <c r="F24" s="33" t="inlineStr"/>
-      <c r="G24" s="33" t="inlineStr"/>
+      <c r="E24" s="36" t="inlineStr"/>
+      <c r="F24" s="36" t="inlineStr"/>
+      <c r="G24" s="36" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="18" t="inlineStr">
@@ -1646,44 +1665,44 @@
       <c r="F28" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="20" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr">
         <is>
           <t>Bridge construction — low margin</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="C29" s="28" t="inlineStr"/>
-      <c r="D29" s="29">
+      <c r="C29" s="31" t="inlineStr"/>
+      <c r="D29" s="32">
         <f>MEDIAN(D28)</f>
         <v/>
       </c>
-      <c r="E29" s="28" t="inlineStr"/>
-      <c r="F29" s="28" t="inlineStr"/>
-      <c r="G29" s="28" t="inlineStr"/>
+      <c r="E29" s="31" t="inlineStr"/>
+      <c r="F29" s="31" t="inlineStr"/>
+      <c r="G29" s="31" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="B30" s="30" t="inlineStr">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>Selected Multiple</t>
         </is>
       </c>
-      <c r="C30" s="31" t="inlineStr">
+      <c r="C30" s="34" t="inlineStr">
         <is>
           <t>Infrastructure floor</t>
         </is>
       </c>
-      <c r="D30" s="32" t="n">
+      <c r="D30" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="E30" s="33" t="inlineStr"/>
-      <c r="F30" s="33" t="inlineStr"/>
-      <c r="G30" s="33" t="inlineStr"/>
+      <c r="E30" s="36" t="inlineStr"/>
+      <c r="F30" s="36" t="inlineStr"/>
+      <c r="G30" s="36" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1773,26 +1792,26 @@
           <t>Aero, Space &amp; Defense</t>
         </is>
       </c>
-      <c r="C5" s="34">
+      <c r="C5" s="37">
         <f>'Segment Data'!E7</f>
         <v/>
       </c>
-      <c r="D5" s="35" t="n">
+      <c r="D5" s="38" t="n">
         <v>0.31</v>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="39">
         <f>B12*D5</f>
         <v/>
       </c>
-      <c r="F5" s="36">
+      <c r="F5" s="39">
         <f>C5+E5</f>
         <v/>
       </c>
-      <c r="G5" s="37">
+      <c r="G5" s="40">
         <f>'Peer Comps'!D10</f>
         <v/>
       </c>
-      <c r="H5" s="36">
+      <c r="H5" s="39">
         <f>F5*G5</f>
         <v/>
       </c>
@@ -1803,26 +1822,26 @@
           <t>Resources, Energy &amp; Environment</t>
         </is>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="37">
         <f>'Segment Data'!E12</f>
         <v/>
       </c>
-      <c r="D6" s="35" t="n">
+      <c r="D6" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="E6" s="36">
+      <c r="E6" s="39">
         <f>B12*D6</f>
         <v/>
       </c>
-      <c r="F6" s="36">
+      <c r="F6" s="39">
         <f>C6+E6</f>
         <v/>
       </c>
-      <c r="G6" s="37">
+      <c r="G6" s="40">
         <f>'Peer Comps'!D17</f>
         <v/>
       </c>
-      <c r="H6" s="36">
+      <c r="H6" s="39">
         <f>F6*G6</f>
         <v/>
       </c>
@@ -1833,26 +1852,26 @@
           <t>Industrial Systems &amp; General Machinery</t>
         </is>
       </c>
-      <c r="C7" s="34">
+      <c r="C7" s="37">
         <f>'Segment Data'!E17</f>
         <v/>
       </c>
-      <c r="D7" s="35" t="n">
+      <c r="D7" s="38" t="n">
         <v>0.27</v>
       </c>
-      <c r="E7" s="36">
+      <c r="E7" s="39">
         <f>B12*D7</f>
         <v/>
       </c>
-      <c r="F7" s="36">
+      <c r="F7" s="39">
         <f>C7+E7</f>
         <v/>
       </c>
-      <c r="G7" s="37">
+      <c r="G7" s="40">
         <f>'Peer Comps'!D24</f>
         <v/>
       </c>
-      <c r="H7" s="36">
+      <c r="H7" s="39">
         <f>F7*G7</f>
         <v/>
       </c>
@@ -1863,26 +1882,26 @@
           <t>Social Infrastructure</t>
         </is>
       </c>
-      <c r="C8" s="34">
+      <c r="C8" s="37">
         <f>'Segment Data'!E22</f>
         <v/>
       </c>
-      <c r="D8" s="35" t="n">
+      <c r="D8" s="38" t="n">
         <v>0.12</v>
       </c>
-      <c r="E8" s="36">
+      <c r="E8" s="39">
         <f>B12*D8</f>
         <v/>
       </c>
-      <c r="F8" s="36">
+      <c r="F8" s="39">
         <f>C8+E8</f>
         <v/>
       </c>
-      <c r="G8" s="37">
+      <c r="G8" s="40">
         <f>'Peer Comps'!D30</f>
         <v/>
       </c>
-      <c r="H8" s="36">
+      <c r="H8" s="39">
         <f>F8*G8</f>
         <v/>
       </c>
@@ -1893,41 +1912,41 @@
           <t>Equity Method Investments</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="41" t="n">
         <v>6200</v>
       </c>
-      <c r="D9" s="39" t="inlineStr"/>
-      <c r="E9" s="39" t="inlineStr"/>
-      <c r="F9" s="36">
+      <c r="D9" s="42" t="inlineStr"/>
+      <c r="E9" s="42" t="inlineStr"/>
+      <c r="F9" s="39">
         <f>C9</f>
         <v/>
       </c>
       <c r="G9" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="39">
         <f>F9*G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>Total Segment EV</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr"/>
-      <c r="D10" s="41" t="inlineStr"/>
-      <c r="E10" s="41" t="inlineStr"/>
-      <c r="F10" s="41" t="inlineStr"/>
-      <c r="G10" s="41" t="inlineStr"/>
-      <c r="H10" s="42">
+      <c r="C10" s="44" t="inlineStr"/>
+      <c r="D10" s="44" t="inlineStr"/>
+      <c r="E10" s="44" t="inlineStr"/>
+      <c r="F10" s="44" t="inlineStr"/>
+      <c r="G10" s="44" t="inlineStr"/>
+      <c r="H10" s="45">
         <f>H5+H6+H7+H8+H9</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="43" t="n">
+      <c r="B12" s="46" t="n">
         <v>70000</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -1949,7 +1968,7 @@
           <t xml:space="preserve">  Aero, Space &amp; Defense</t>
         </is>
       </c>
-      <c r="C15" s="44">
+      <c r="C15" s="47">
         <f>H5/H10</f>
         <v/>
       </c>
@@ -1960,7 +1979,7 @@
           <t xml:space="preserve">  Resources, Energy &amp; Environment</t>
         </is>
       </c>
-      <c r="C16" s="44">
+      <c r="C16" s="47">
         <f>H6/H10</f>
         <v/>
       </c>
@@ -1971,7 +1990,7 @@
           <t xml:space="preserve">  Industrial Systems &amp; General Machinery</t>
         </is>
       </c>
-      <c r="C17" s="44">
+      <c r="C17" s="47">
         <f>H7/H10</f>
         <v/>
       </c>
@@ -1982,7 +2001,7 @@
           <t xml:space="preserve">  Social Infrastructure</t>
         </is>
       </c>
-      <c r="C18" s="44">
+      <c r="C18" s="47">
         <f>H8/H10</f>
         <v/>
       </c>
@@ -2001,7 +2020,7 @@
           <t>Total Enterprise Value</t>
         </is>
       </c>
-      <c r="C21" s="34">
+      <c r="C21" s="37">
         <f>H10</f>
         <v/>
       </c>
@@ -2012,7 +2031,7 @@
           <t>Conglomerate Discount</t>
         </is>
       </c>
-      <c r="C22" s="45" t="n">
+      <c r="C22" s="48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2022,7 +2041,7 @@
           <t>Adjusted EV</t>
         </is>
       </c>
-      <c r="C23" s="36">
+      <c r="C23" s="39">
         <f>C21*(1-C22)</f>
         <v/>
       </c>
@@ -2048,12 +2067,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="27" t="inlineStr">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Equity Value</t>
         </is>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="49">
         <f>C23-C24-C25</f>
         <v/>
       </c>
@@ -2064,7 +2083,7 @@
           <t>Shares Outstanding (thousands)</t>
         </is>
       </c>
-      <c r="C27" s="47" t="n">
+      <c r="C27" s="50" t="n">
         <v>151364</v>
       </c>
     </row>
@@ -2074,17 +2093,17 @@
           <t>Stock Split Ratio</t>
         </is>
       </c>
-      <c r="C28" s="47" t="n">
+      <c r="C28" s="50" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="48" t="inlineStr">
+      <c r="B29" s="51" t="inlineStr">
         <is>
           <t>Fair Value Per Share (post-split)</t>
         </is>
       </c>
-      <c r="C29" s="49">
+      <c r="C29" s="52">
         <f>C26*1000/C27/C28</f>
         <v/>
       </c>
@@ -2108,7 +2127,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -2151,19 +2170,19 @@
           <t>Aero, Space &amp; Defense OP</t>
         </is>
       </c>
-      <c r="C6" s="50">
+      <c r="C6" s="53">
         <f>'SOTP Valuation'!C5</f>
         <v/>
       </c>
-      <c r="D6" s="50">
+      <c r="D6" s="53">
         <f>'SOTP Valuation'!E5</f>
         <v/>
       </c>
-      <c r="E6" s="51">
+      <c r="E6" s="54">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="52">
+      <c r="F6" s="55">
         <f>'SOTP Valuation'!G5</f>
         <v/>
       </c>
@@ -2174,19 +2193,19 @@
           <t>Resources, Energy &amp; Environment OP</t>
         </is>
       </c>
-      <c r="C7" s="50">
+      <c r="C7" s="53">
         <f>'SOTP Valuation'!C6</f>
         <v/>
       </c>
-      <c r="D7" s="50">
+      <c r="D7" s="53">
         <f>'SOTP Valuation'!E6</f>
         <v/>
       </c>
-      <c r="E7" s="51">
+      <c r="E7" s="54">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="52">
+      <c r="F7" s="55">
         <f>'SOTP Valuation'!G6</f>
         <v/>
       </c>
@@ -2197,19 +2216,19 @@
           <t>Industrial Systems &amp; General Machinery OP</t>
         </is>
       </c>
-      <c r="C8" s="50">
+      <c r="C8" s="53">
         <f>'SOTP Valuation'!C7</f>
         <v/>
       </c>
-      <c r="D8" s="50">
+      <c r="D8" s="53">
         <f>'SOTP Valuation'!E7</f>
         <v/>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="54">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="52">
+      <c r="F8" s="55">
         <f>'SOTP Valuation'!G7</f>
         <v/>
       </c>
@@ -2220,19 +2239,19 @@
           <t>Social Infrastructure OP</t>
         </is>
       </c>
-      <c r="C9" s="50">
+      <c r="C9" s="53">
         <f>'SOTP Valuation'!C8</f>
         <v/>
       </c>
-      <c r="D9" s="50">
+      <c r="D9" s="53">
         <f>'SOTP Valuation'!E8</f>
         <v/>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="54">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="55">
         <f>'SOTP Valuation'!G8</f>
         <v/>
       </c>
@@ -2243,7 +2262,7 @@
           <t>Equity Method EV</t>
         </is>
       </c>
-      <c r="C10" s="50">
+      <c r="C10" s="53">
         <f>'SOTP Valuation'!H9</f>
         <v/>
       </c>
@@ -2254,7 +2273,7 @@
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="C11" s="50">
+      <c r="C11" s="53">
         <f>'SOTP Valuation'!C24</f>
         <v/>
       </c>
@@ -2265,7 +2284,7 @@
           <t>Minority Interest</t>
         </is>
       </c>
-      <c r="C12" s="50">
+      <c r="C12" s="53">
         <f>'SOTP Valuation'!C25</f>
         <v/>
       </c>
@@ -2276,7 +2295,7 @@
           <t>Shares (thousands)</t>
         </is>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="56">
         <f>'SOTP Valuation'!C27</f>
         <v/>
       </c>
@@ -2287,7 +2306,7 @@
           <t>Split Ratio</t>
         </is>
       </c>
-      <c r="C14" s="53">
+      <c r="C14" s="56">
         <f>'SOTP Valuation'!C28</f>
         <v/>
       </c>
@@ -2298,166 +2317,166 @@
           <t>Aero, Space &amp; Defense EV/EBITDA →</t>
         </is>
       </c>
-      <c r="C16" s="54" t="n">
+      <c r="C16" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="D16" s="54" t="n">
+      <c r="D16" s="57" t="n">
         <v>16</v>
       </c>
-      <c r="E16" s="54" t="n">
+      <c r="E16" s="57" t="n">
         <v>18</v>
       </c>
-      <c r="F16" s="54" t="n">
+      <c r="F16" s="57" t="n">
         <v>20</v>
       </c>
-      <c r="G16" s="54" t="n">
+      <c r="G16" s="57" t="n">
         <v>22</v>
       </c>
-      <c r="H16" s="54" t="n">
+      <c r="H16" s="57" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="55" t="n">
+      <c r="B17" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="59">
         <f>(($E$6*14+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="59">
         <f>(($E$6*16+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E17" s="57">
+      <c r="E17" s="60">
         <f>(($E$6*18+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F17" s="56">
+      <c r="F17" s="59">
         <f>(($E$6*20+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="G17" s="56">
+      <c r="G17" s="59">
         <f>(($E$6*22+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="H17" s="56">
+      <c r="H17" s="59">
         <f>(($E$6*25+E7*F7+E8*F8+E9*F9+C10)*(1-$B17)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="55" t="n">
+      <c r="B18" s="58" t="n">
         <v>0.05</v>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="59">
         <f>(($E$6*14+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D18" s="56">
+      <c r="D18" s="59">
         <f>(($E$6*16+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E18" s="56">
+      <c r="E18" s="59">
         <f>(($E$6*18+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F18" s="56">
+      <c r="F18" s="59">
         <f>(($E$6*20+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="G18" s="56">
+      <c r="G18" s="59">
         <f>(($E$6*22+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="H18" s="56">
+      <c r="H18" s="59">
         <f>(($E$6*25+E7*F7+E8*F8+E9*F9+C10)*(1-$B18)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="55" t="n">
+      <c r="B19" s="58" t="n">
         <v>0.1</v>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="59">
         <f>(($E$6*14+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D19" s="56">
+      <c r="D19" s="59">
         <f>(($E$6*16+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E19" s="56">
+      <c r="E19" s="59">
         <f>(($E$6*18+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F19" s="56">
+      <c r="F19" s="59">
         <f>(($E$6*20+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="G19" s="56">
+      <c r="G19" s="59">
         <f>(($E$6*22+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="H19" s="56">
+      <c r="H19" s="59">
         <f>(($E$6*25+E7*F7+E8*F8+E9*F9+C10)*(1-$B19)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="55" t="n">
+      <c r="B20" s="58" t="n">
         <v>0.15</v>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="59">
         <f>(($E$6*14+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="59">
         <f>(($E$6*16+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E20" s="56">
+      <c r="E20" s="59">
         <f>(($E$6*18+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F20" s="56">
+      <c r="F20" s="59">
         <f>(($E$6*20+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="G20" s="56">
+      <c r="G20" s="59">
         <f>(($E$6*22+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="H20" s="56">
+      <c r="H20" s="59">
         <f>(($E$6*25+E7*F7+E8*F8+E9*F9+C10)*(1-$B20)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="55" t="n">
+      <c r="B21" s="58" t="n">
         <v>0.2</v>
       </c>
-      <c r="C21" s="56">
+      <c r="C21" s="59">
         <f>(($E$6*14+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D21" s="56">
+      <c r="D21" s="59">
         <f>(($E$6*16+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E21" s="56">
+      <c r="E21" s="59">
         <f>(($E$6*18+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F21" s="56">
+      <c r="F21" s="59">
         <f>(($E$6*20+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="G21" s="56">
+      <c r="G21" s="59">
         <f>(($E$6*22+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="H21" s="56">
+      <c r="H21" s="59">
         <f>(($E$6*25+E7*F7+E8*F8+E9*F9+C10)*(1-$B21)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
@@ -2482,120 +2501,120 @@
           <t>Industrial Systems &amp; General Machinery ↓ / Resources, Energy &amp; Environment →</t>
         </is>
       </c>
-      <c r="C26" s="54" t="n">
+      <c r="C26" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="D26" s="54" t="n">
+      <c r="D26" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="E26" s="54" t="n">
+      <c r="E26" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="F26" s="54" t="n">
+      <c r="F26" s="57" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="58" t="n">
+      <c r="B27" s="61" t="n">
         <v>7</v>
       </c>
-      <c r="C27" s="56">
+      <c r="C27" s="59">
         <f>(($E$8*$B27+$E$7*C$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D27" s="56">
+      <c r="D27" s="59">
         <f>(($E$8*$B27+$E$7*D$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E27" s="56">
+      <c r="E27" s="59">
         <f>(($E$8*$B27+$E$7*E$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F27" s="56">
+      <c r="F27" s="59">
         <f>(($E$8*$B27+$E$7*F$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="58" t="n">
+      <c r="B28" s="61" t="n">
         <v>8</v>
       </c>
-      <c r="C28" s="56">
+      <c r="C28" s="59">
         <f>(($E$8*$B28+$E$7*C$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D28" s="56">
+      <c r="D28" s="59">
         <f>(($E$8*$B28+$E$7*D$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E28" s="56">
+      <c r="E28" s="59">
         <f>(($E$8*$B28+$E$7*E$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F28" s="56">
+      <c r="F28" s="59">
         <f>(($E$8*$B28+$E$7*F$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="58" t="n">
+      <c r="B29" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="C29" s="56">
+      <c r="C29" s="59">
         <f>(($E$8*$B29+$E$7*C$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D29" s="57">
+      <c r="D29" s="60">
         <f>(($E$8*$B29+$E$7*D$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E29" s="56">
+      <c r="E29" s="59">
         <f>(($E$8*$B29+$E$7*E$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F29" s="56">
+      <c r="F29" s="59">
         <f>(($E$8*$B29+$E$7*F$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="58" t="n">
+      <c r="B30" s="61" t="n">
         <v>12</v>
       </c>
-      <c r="C30" s="56">
+      <c r="C30" s="59">
         <f>(($E$8*$B30+$E$7*C$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D30" s="56">
+      <c r="D30" s="59">
         <f>(($E$8*$B30+$E$7*D$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E30" s="56">
+      <c r="E30" s="59">
         <f>(($E$8*$B30+$E$7*E$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F30" s="56">
+      <c r="F30" s="59">
         <f>(($E$8*$B30+$E$7*F$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="58" t="n">
+      <c r="B31" s="61" t="n">
         <v>14</v>
       </c>
-      <c r="C31" s="56">
+      <c r="C31" s="59">
         <f>(($E$8*$B31+$E$7*C$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="D31" s="56">
+      <c r="D31" s="59">
         <f>(($E$8*$B31+$E$7*D$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="E31" s="56">
+      <c r="E31" s="59">
         <f>(($E$8*$B31+$E$7*E$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
-      <c r="F31" s="56">
+      <c r="F31" s="59">
         <f>(($E$8*$B31+$E$7*F$26+$E$6*$F$6+$E$9*$F$9+$C$10)*(1-0.0)-$C$11-$C$12)*1000/$C$13/$C$14</f>
         <v/>
       </c>
@@ -2649,7 +2668,7 @@
           <t>Consolidated D&amp;A (FY25E)</t>
         </is>
       </c>
-      <c r="C6" s="43" t="n">
+      <c r="C6" s="46" t="n">
         <v>70000</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -2686,10 +2705,10 @@
           <t>Aero, Space &amp; Defense</t>
         </is>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="38" t="n">
         <v>0.31</v>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="39">
         <f>$C$6*C9</f>
         <v/>
       </c>
@@ -2700,10 +2719,10 @@
           <t>Resources, Energy &amp; Environment</t>
         </is>
       </c>
-      <c r="C10" s="35" t="n">
+      <c r="C10" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="39">
         <f>$C$6*C10</f>
         <v/>
       </c>
@@ -2714,10 +2733,10 @@
           <t>Industrial Systems &amp; General Machinery</t>
         </is>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="C11" s="38" t="n">
         <v>0.27</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="39">
         <f>$C$6*C11</f>
         <v/>
       </c>
@@ -2728,29 +2747,29 @@
           <t>Social Infrastructure</t>
         </is>
       </c>
-      <c r="C12" s="35" t="n">
+      <c r="C12" s="38" t="n">
         <v>0.12</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="39">
         <f>$C$6*C12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="40" t="inlineStr">
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C13" s="59">
+      <c r="C13" s="62">
         <f>C9+C10+C11+C12</f>
         <v/>
       </c>
-      <c r="D13" s="42">
+      <c r="D13" s="45">
         <f>D9+D10+D11+D12</f>
         <v/>
       </c>
-      <c r="E13" s="40">
+      <c r="E13" s="43">
         <f>IF(ABS(C13-1)&lt;0.001,"OK","CHECK")</f>
         <v/>
       </c>

</xml_diff>